<commit_message>
Atualizando o banco de exemplo para a versao 4 e os xlsx processados com a aba meteorologia_15min
</commit_message>
<xml_diff>
--- a/dados/processados/integracao_usina_20260922.xlsx
+++ b/dados/processados/integracao_usina_20260922.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="eletrico_5min" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="integracao_15min" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resumo" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="meteorologia_15min" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="resumo" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9751,6 +9752,437 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:CE1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>timestamp_15min</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>timestamp_original</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>lacuna_temporal</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ghi_lppyra02_w_m2</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ghi_lpnet14_w_m2</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>temperatura_c</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>vento_m_s</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>precipitacao</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>umidade_relativa_inst_pct</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>umidade_relativa_med_pct</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>umidade_relativa_max_pct</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>umidade_relativa_min_pct</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>vento_dir_med_graus</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>vento_dir_max_graus</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>vento_dir_min_graus</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>vento_vel_max_m_s</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>vento_vel_min_m_s</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>ghi_lppyra02_med_w_m2</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>ghi_lppyra02_max_w_m2</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>ghi_lppyra02_min_w_m2</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>ghi_lpnet14_med_w_m2</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>ghi_lpnet14_max_w_m2</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>ghi_lpnet14_min_w_m2</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>umid_solo_inst</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>umid_solo_med</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>umid_solo_max</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>umid_solo_min</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>pressao_inst_hpa</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>pressao_med_hpa</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>pressao_max_hpa</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>pressao_min_hpa</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>temp_int_c</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>temperatura_med_c</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>temperatura_max_c</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>temperatura_min_c</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>rad_refletida_inst_w_m2</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>rad_refletida_med_w_m2</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>rad_refletida_max_w_m2</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>rad_refletida_min_w_m2</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>rad_iv_inst_w_m2</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>rad_iv_med_w_m2</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>rad_iv_max_w_m2</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>rad_iv_min_w_m2</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>rad_spf_inst_w_m2</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>rad_spf_med_w_m2</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>rad_spf_max_w_m2</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>rad_spf_min_w_m2</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>rad_liquida_inst_w_m2</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>rad_liquida_med_w_m2</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>rad_liquida_max_w_m2</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>rad_liquida_min_w_m2</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>temp_ntc_lpnet14_inst_c</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>temp_ntc_lpnet14_med_c</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>temp_ntc_lpnet14_max_c</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>temp_ntc_lpnet14_min_c</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>temp_solo_inst</t>
+        </is>
+      </c>
+      <c r="BE1" t="inlineStr">
+        <is>
+          <t>temp_solo_med</t>
+        </is>
+      </c>
+      <c r="BF1" t="inlineStr">
+        <is>
+          <t>temp_solo_max</t>
+        </is>
+      </c>
+      <c r="BG1" t="inlineStr">
+        <is>
+          <t>temp_solo_min</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
+          <t>flag_ghi_lppyra02_w_m2</t>
+        </is>
+      </c>
+      <c r="BI1" t="inlineStr">
+        <is>
+          <t>flag_ghi_lpnet14_w_m2</t>
+        </is>
+      </c>
+      <c r="BJ1" t="inlineStr">
+        <is>
+          <t>flag_temperatura_c</t>
+        </is>
+      </c>
+      <c r="BK1" t="inlineStr">
+        <is>
+          <t>flag_vento_m_s</t>
+        </is>
+      </c>
+      <c r="BL1" t="inlineStr">
+        <is>
+          <t>flag_precipitacao</t>
+        </is>
+      </c>
+      <c r="BM1" t="inlineStr">
+        <is>
+          <t>flag_umidade_relativa_inst_pct</t>
+        </is>
+      </c>
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>flag_umidade_relativa_med_pct</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>flag_umidade_relativa_max_pct</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>flag_umidade_relativa_min_pct</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>flag_vento_dir_med_graus</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>flag_vento_dir_max_graus</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>flag_vento_dir_min_graus</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>flag_vento_vel_max_m_s</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>flag_vento_vel_min_m_s</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>flag_ghi_lppyra02_med_w_m2</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>flag_ghi_lppyra02_max_w_m2</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>flag_ghi_lppyra02_min_w_m2</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
+          <t>flag_ghi_lpnet14_med_w_m2</t>
+        </is>
+      </c>
+      <c r="BZ1" t="inlineStr">
+        <is>
+          <t>flag_ghi_lpnet14_max_w_m2</t>
+        </is>
+      </c>
+      <c r="CA1" t="inlineStr">
+        <is>
+          <t>flag_ghi_lpnet14_min_w_m2</t>
+        </is>
+      </c>
+      <c r="CB1" t="inlineStr">
+        <is>
+          <t>flag_umid_solo_inst</t>
+        </is>
+      </c>
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>flag_umid_solo_med</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr">
+        <is>
+          <t>flag_umid_solo_max</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr">
+        <is>
+          <t>flag_umid_solo_min</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>